<commit_message>
Working site pre-image captions
</commit_message>
<xml_diff>
--- a/epcot_wait_times.xlsx
+++ b/epcot_wait_times.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hrhpi\Documents\GitHub\disney-wait-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2933C2D2-0D39-452C-9A75-DAE88795B4B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF01B70-C7A2-44A4-AF9F-559F142C97E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2A99A6C3-3396-4AE7-88F2-C04D38FA5BF3}"/>
   </bookViews>
@@ -548,10 +548,10 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -560,7 +560,7 @@
         <v>5</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I1" t="s">
         <v>26</v>
@@ -576,11 +576,11 @@
       <c r="C2" t="s">
         <v>25</v>
       </c>
-      <c r="D2">
-        <v>49</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="D2" t="s">
         <v>25</v>
+      </c>
+      <c r="E2">
+        <v>73</v>
       </c>
       <c r="F2">
         <v>75</v>
@@ -589,7 +589,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="I2">
         <v>60</v>
@@ -606,10 +606,10 @@
         <v>49</v>
       </c>
       <c r="D3">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="E3">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F3">
         <v>73</v>
@@ -618,7 +618,7 @@
         <v>45</v>
       </c>
       <c r="H3">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="I3">
         <v>36</v>
@@ -635,10 +635,10 @@
         <v>61</v>
       </c>
       <c r="D4">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="E4">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F4">
         <v>56</v>
@@ -647,7 +647,7 @@
         <v>42</v>
       </c>
       <c r="H4">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="I4">
         <v>15</v>
@@ -664,10 +664,10 @@
         <v>59</v>
       </c>
       <c r="D5">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="E5">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F5">
         <v>52</v>
@@ -676,7 +676,7 @@
         <v>25</v>
       </c>
       <c r="H5">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="I5">
         <v>13</v>
@@ -692,11 +692,11 @@
       <c r="C6">
         <v>42</v>
       </c>
-      <c r="D6" t="s">
-        <v>25</v>
+      <c r="D6">
+        <v>39</v>
       </c>
       <c r="E6">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F6">
         <v>43</v>
@@ -704,8 +704,8 @@
       <c r="G6">
         <v>29</v>
       </c>
-      <c r="H6">
-        <v>40</v>
+      <c r="H6" t="s">
+        <v>25</v>
       </c>
       <c r="I6" t="s">
         <v>25</v>
@@ -722,10 +722,10 @@
         <v>41</v>
       </c>
       <c r="D7">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="E7">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F7">
         <v>33</v>
@@ -734,7 +734,7 @@
         <v>10</v>
       </c>
       <c r="H7">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="I7">
         <v>13</v>
@@ -751,10 +751,10 @@
         <v>17</v>
       </c>
       <c r="D8">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E8">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F8">
         <v>19</v>
@@ -763,7 +763,7 @@
         <v>14</v>
       </c>
       <c r="H8">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="I8">
         <v>15</v>
@@ -780,7 +780,7 @@
         <v>26</v>
       </c>
       <c r="D9">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="E9">
         <v>21</v>
@@ -792,7 +792,7 @@
         <v>25</v>
       </c>
       <c r="H9">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="I9">
         <v>30</v>
@@ -809,10 +809,10 @@
         <v>18</v>
       </c>
       <c r="D10">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E10">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F10">
         <v>17</v>
@@ -821,7 +821,7 @@
         <v>5</v>
       </c>
       <c r="H10">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="I10">
         <v>5</v>
@@ -867,10 +867,10 @@
         <v>14</v>
       </c>
       <c r="D12">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E12">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F12">
         <v>22</v>
@@ -879,7 +879,7 @@
         <v>5</v>
       </c>
       <c r="H12">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I12">
         <v>5</v>
@@ -896,10 +896,10 @@
         <v>21</v>
       </c>
       <c r="D13">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="E13">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F13">
         <v>14</v>
@@ -908,7 +908,7 @@
         <v>5</v>
       </c>
       <c r="H13">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I13">
         <v>5</v>
@@ -925,7 +925,7 @@
         <v>14</v>
       </c>
       <c r="D14">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E14">
         <v>11</v>
@@ -937,7 +937,7 @@
         <v>25</v>
       </c>
       <c r="H14">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="I14">
         <v>5</v>
@@ -954,10 +954,10 @@
         <v>18</v>
       </c>
       <c r="D15">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E15">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F15">
         <v>8</v>
@@ -966,7 +966,7 @@
         <v>25</v>
       </c>
       <c r="H15">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I15">
         <v>6</v>

</xml_diff>

<commit_message>
Code cleanup and final changes
</commit_message>
<xml_diff>
--- a/epcot_wait_times.xlsx
+++ b/epcot_wait_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hrhpi\Documents\GitHub\disney-wait-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF01B70-C7A2-44A4-AF9F-559F142C97E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BB9223F-2613-4285-A0B9-FD51936B7809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2A99A6C3-3396-4AE7-88F2-C04D38FA5BF3}"/>
+    <workbookView xWindow="7200" yWindow="4155" windowWidth="21600" windowHeight="11295" xr2:uid="{2A99A6C3-3396-4AE7-88F2-C04D38FA5BF3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,9 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
   <si>
-    <t>Average</t>
-  </si>
-  <si>
     <t>Festival of the Arts</t>
   </si>
   <si>
@@ -153,6 +150,9 @@
   </si>
   <si>
     <t>December</t>
+  </si>
+  <si>
+    <t>2025 Average</t>
   </si>
 </sst>
 </file>
@@ -539,45 +539,45 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>2</v>
-      </c>
       <c r="I1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2">
         <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2">
         <v>73</v>
@@ -597,7 +597,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>60</v>
@@ -626,7 +626,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>46</v>
@@ -655,7 +655,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5">
         <v>38</v>
@@ -684,7 +684,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6">
         <v>39</v>
@@ -705,15 +705,15 @@
         <v>29</v>
       </c>
       <c r="H6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7">
         <v>20</v>
@@ -742,7 +742,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8">
         <v>17</v>
@@ -771,7 +771,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9">
         <v>23</v>
@@ -789,7 +789,7 @@
         <v>23</v>
       </c>
       <c r="G9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H9">
         <v>29</v>
@@ -800,7 +800,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10">
         <v>10</v>
@@ -829,7 +829,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B11">
         <v>15</v>
@@ -853,12 +853,12 @@
         <v>15</v>
       </c>
       <c r="I11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B12">
         <v>9</v>
@@ -887,7 +887,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B13">
         <v>10</v>
@@ -916,7 +916,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14">
         <v>10</v>
@@ -934,7 +934,7 @@
         <v>9</v>
       </c>
       <c r="G14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H14">
         <v>6</v>
@@ -945,7 +945,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B15">
         <v>9</v>
@@ -963,7 +963,7 @@
         <v>8</v>
       </c>
       <c r="G15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H15">
         <v>6</v>
@@ -974,15 +974,15 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18">
         <v>66</v>
@@ -990,7 +990,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19">
         <v>65</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20">
         <v>67</v>
@@ -1006,7 +1006,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21">
         <v>48</v>
@@ -1014,7 +1014,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22">
         <v>48</v>
@@ -1022,7 +1022,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B23">
         <v>31</v>
@@ -1030,7 +1030,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24">
         <v>28</v>
@@ -1038,7 +1038,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25">
         <v>28</v>
@@ -1046,7 +1046,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B26">
         <v>41</v>
@@ -1054,7 +1054,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B27">
         <v>49</v>
@@ -1062,7 +1062,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B28">
         <v>53</v>
@@ -1070,7 +1070,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B29">
         <v>56</v>

</xml_diff>